<commit_message>
Cross-check franchise list against legacy Core Assortment FW27 flag
Adds two columns: the pre-Tobias-data Core Assortment FW27 flag from the
SS26 tiering workbook (rolled up to Base grain), and whether it agrees
with the new FW27/SS28 data's Active flag. Scoped the comparison to only
the 34 Yes/Mixed legacy franchises, since the legacy flag is a narrow
strategic-item signal, not a full range flag -- comparing it against all
258 franchises produced noise, not findings.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bz4WiqJXGrQWfCc7f9Cm8G
</commit_message>
<xml_diff>
--- a/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
+++ b/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Notes" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Franchise Review List'!$A$1:$L$259</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Franchise Review List'!$A$1:$N$259</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L259"/>
+  <dimension ref="A1:N259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -444,6 +444,8 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="29" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,6 +507,16 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t># styles rolled up</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Legacy Core Assortment FW27</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Agrees with new FW27-active?</t>
         </is>
       </c>
     </row>
@@ -545,6 +557,12 @@
       <c r="L2" t="n">
         <v>1</v>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -583,6 +601,16 @@
       <c r="L3" t="n">
         <v>1</v>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -625,6 +653,16 @@
       <c r="L4" t="n">
         <v>2</v>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -667,6 +705,12 @@
       <c r="L5" t="n">
         <v>2</v>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -705,6 +749,12 @@
       <c r="L6" t="n">
         <v>1</v>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -743,6 +793,12 @@
       <c r="L7" t="n">
         <v>1</v>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -781,6 +837,12 @@
       <c r="L8" t="n">
         <v>1</v>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -819,6 +881,12 @@
       <c r="L9" t="n">
         <v>1</v>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -861,6 +929,12 @@
       <c r="L10" t="n">
         <v>2</v>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -899,6 +973,12 @@
       <c r="L11" t="n">
         <v>1</v>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -937,6 +1017,12 @@
       <c r="L12" t="n">
         <v>1</v>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -975,6 +1061,12 @@
       <c r="L13" t="n">
         <v>1</v>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1013,6 +1105,12 @@
       <c r="L14" t="n">
         <v>1</v>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1051,6 +1149,12 @@
       <c r="L15" t="n">
         <v>1</v>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1093,6 +1197,12 @@
       <c r="L16" t="n">
         <v>2</v>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1131,6 +1241,12 @@
       <c r="L17" t="n">
         <v>1</v>
       </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1169,6 +1285,12 @@
       <c r="L18" t="n">
         <v>1</v>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1207,6 +1329,12 @@
       <c r="L19" t="n">
         <v>1</v>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1245,6 +1373,12 @@
       <c r="L20" t="n">
         <v>1</v>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1283,6 +1417,12 @@
       <c r="L21" t="n">
         <v>1</v>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1321,6 +1461,12 @@
       <c r="L22" t="n">
         <v>1</v>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1369,6 +1515,12 @@
       <c r="L23" t="n">
         <v>2</v>
       </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1411,6 +1563,12 @@
       <c r="L24" t="n">
         <v>2</v>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1449,6 +1607,12 @@
       <c r="L25" t="n">
         <v>1</v>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1491,6 +1655,12 @@
       <c r="L26" t="n">
         <v>2</v>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1533,6 +1703,12 @@
       <c r="L27" t="n">
         <v>2</v>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1575,6 +1751,12 @@
       <c r="L28" t="n">
         <v>2</v>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1617,6 +1799,12 @@
       <c r="L29" t="n">
         <v>2</v>
       </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1659,6 +1847,12 @@
       <c r="L30" t="n">
         <v>2</v>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1701,6 +1895,12 @@
       <c r="L31" t="n">
         <v>2</v>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1743,6 +1943,12 @@
       <c r="L32" t="n">
         <v>2</v>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1785,6 +1991,12 @@
       <c r="L33" t="n">
         <v>2</v>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1827,6 +2039,12 @@
       <c r="L34" t="n">
         <v>2</v>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1869,6 +2087,12 @@
       <c r="L35" t="n">
         <v>2</v>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1911,6 +2135,12 @@
       <c r="L36" t="n">
         <v>2</v>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1957,6 +2187,12 @@
       <c r="L37" t="n">
         <v>3</v>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1999,6 +2235,16 @@
       <c r="L38" t="n">
         <v>2</v>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2041,6 +2287,16 @@
       <c r="L39" t="n">
         <v>2</v>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2083,6 +2339,12 @@
       <c r="L40" t="n">
         <v>2</v>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2125,6 +2387,12 @@
       <c r="L41" t="n">
         <v>2</v>
       </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2167,6 +2435,12 @@
       <c r="L42" t="n">
         <v>2</v>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2209,6 +2483,12 @@
       <c r="L43" t="n">
         <v>2</v>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2251,6 +2531,12 @@
       <c r="L44" t="n">
         <v>2</v>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2293,6 +2579,12 @@
       <c r="L45" t="n">
         <v>2</v>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2335,6 +2627,16 @@
       <c r="L46" t="n">
         <v>2</v>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2377,6 +2679,12 @@
       <c r="L47" t="n">
         <v>2</v>
       </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2419,6 +2727,12 @@
       <c r="L48" t="n">
         <v>2</v>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2461,6 +2775,12 @@
       <c r="L49" t="n">
         <v>2</v>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2503,6 +2823,12 @@
       <c r="L50" t="n">
         <v>2</v>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2545,6 +2871,12 @@
       <c r="L51" t="n">
         <v>2</v>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2583,6 +2915,12 @@
       <c r="L52" t="n">
         <v>2</v>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2621,6 +2959,12 @@
       <c r="L53" t="n">
         <v>2</v>
       </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2659,6 +3003,12 @@
       <c r="L54" t="n">
         <v>2</v>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2697,6 +3047,12 @@
       <c r="L55" t="n">
         <v>2</v>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2739,6 +3095,12 @@
       <c r="L56" t="n">
         <v>2</v>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2781,6 +3143,16 @@
       <c r="L57" t="n">
         <v>2</v>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2823,6 +3195,16 @@
       <c r="L58" t="n">
         <v>2</v>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2865,6 +3247,12 @@
       <c r="L59" t="n">
         <v>2</v>
       </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2907,6 +3295,12 @@
       <c r="L60" t="n">
         <v>2</v>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2949,6 +3343,12 @@
       <c r="L61" t="n">
         <v>2</v>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2995,6 +3395,12 @@
       <c r="L62" t="n">
         <v>2</v>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3041,6 +3447,12 @@
       <c r="L63" t="n">
         <v>2</v>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3083,6 +3495,16 @@
       <c r="L64" t="n">
         <v>2</v>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3128,6 +3550,16 @@
       </c>
       <c r="L65" t="n">
         <v>3</v>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -3171,6 +3603,12 @@
       <c r="L66" t="n">
         <v>2</v>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3213,6 +3651,12 @@
       <c r="L67" t="n">
         <v>2</v>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3255,6 +3699,12 @@
       <c r="L68" t="n">
         <v>2</v>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3297,6 +3747,12 @@
       <c r="L69" t="n">
         <v>2</v>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3339,6 +3795,12 @@
       <c r="L70" t="n">
         <v>2</v>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3381,6 +3843,12 @@
       <c r="L71" t="n">
         <v>2</v>
       </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3423,6 +3891,12 @@
       <c r="L72" t="n">
         <v>2</v>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3465,6 +3939,12 @@
       <c r="L73" t="n">
         <v>2</v>
       </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3507,6 +3987,12 @@
       <c r="L74" t="n">
         <v>2</v>
       </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3549,6 +4035,12 @@
       <c r="L75" t="n">
         <v>2</v>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3591,6 +4083,12 @@
       <c r="L76" t="n">
         <v>2</v>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3633,6 +4131,12 @@
       <c r="L77" t="n">
         <v>2</v>
       </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3675,6 +4179,12 @@
       <c r="L78" t="n">
         <v>2</v>
       </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3717,6 +4227,12 @@
       <c r="L79" t="n">
         <v>2</v>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -3759,6 +4275,12 @@
       <c r="L80" t="n">
         <v>4</v>
       </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -3801,6 +4323,12 @@
       <c r="L81" t="n">
         <v>4</v>
       </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3839,6 +4367,12 @@
       <c r="L82" t="n">
         <v>2</v>
       </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3881,6 +4415,12 @@
       <c r="L83" t="n">
         <v>4</v>
       </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3923,6 +4463,12 @@
       <c r="L84" t="n">
         <v>4</v>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3961,6 +4507,12 @@
       <c r="L85" t="n">
         <v>2</v>
       </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4003,6 +4555,16 @@
       <c r="L86" t="n">
         <v>4</v>
       </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4045,6 +4607,12 @@
       <c r="L87" t="n">
         <v>4</v>
       </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4087,6 +4655,12 @@
       <c r="L88" t="n">
         <v>4</v>
       </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4129,6 +4703,12 @@
       <c r="L89" t="n">
         <v>4</v>
       </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4177,6 +4757,12 @@
       <c r="L90" t="n">
         <v>4</v>
       </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4219,6 +4805,12 @@
       <c r="L91" t="n">
         <v>4</v>
       </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4257,6 +4849,12 @@
       <c r="L92" t="n">
         <v>2</v>
       </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4295,6 +4893,12 @@
       <c r="L93" t="n">
         <v>2</v>
       </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4337,6 +4941,12 @@
       <c r="L94" t="n">
         <v>1</v>
       </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4379,6 +4989,16 @@
       <c r="L95" t="n">
         <v>4</v>
       </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -4421,6 +5041,16 @@
       <c r="L96" t="n">
         <v>4</v>
       </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -4459,6 +5089,12 @@
       <c r="L97" t="n">
         <v>2</v>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -4497,6 +5133,12 @@
       <c r="L98" t="n">
         <v>2</v>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4539,6 +5181,12 @@
       <c r="L99" t="n">
         <v>4</v>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4577,6 +5225,12 @@
       <c r="L100" t="n">
         <v>2</v>
       </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -4619,6 +5273,16 @@
       <c r="L101" t="n">
         <v>1</v>
       </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4661,6 +5325,12 @@
       <c r="L102" t="n">
         <v>1</v>
       </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -4703,6 +5373,12 @@
       <c r="L103" t="n">
         <v>4</v>
       </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -4745,6 +5421,16 @@
       <c r="L104" t="n">
         <v>4</v>
       </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -4787,6 +5473,16 @@
       <c r="L105" t="n">
         <v>4</v>
       </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4825,6 +5521,12 @@
       <c r="L106" t="n">
         <v>2</v>
       </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4863,6 +5565,12 @@
       <c r="L107" t="n">
         <v>2</v>
       </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4905,6 +5613,16 @@
       <c r="L108" t="n">
         <v>4</v>
       </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4943,6 +5661,16 @@
       <c r="L109" t="n">
         <v>2</v>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4981,6 +5709,16 @@
       <c r="L110" t="n">
         <v>2</v>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5019,6 +5757,16 @@
       <c r="L111" t="n">
         <v>2</v>
       </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>Mixed by gender</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Y (mixed by gender)</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5057,6 +5805,12 @@
       <c r="L112" t="n">
         <v>2</v>
       </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5095,6 +5849,12 @@
       <c r="L113" t="n">
         <v>2</v>
       </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5133,6 +5893,12 @@
       <c r="L114" t="n">
         <v>2</v>
       </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5175,6 +5941,16 @@
       <c r="L115" t="n">
         <v>4</v>
       </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -5217,6 +5993,16 @@
       <c r="L116" t="n">
         <v>4</v>
       </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -5255,6 +6041,12 @@
       <c r="L117" t="n">
         <v>2</v>
       </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -5297,6 +6089,12 @@
       <c r="L118" t="n">
         <v>1</v>
       </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -5339,6 +6137,12 @@
       <c r="L119" t="n">
         <v>4</v>
       </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -5377,6 +6181,12 @@
       <c r="L120" t="n">
         <v>2</v>
       </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -5415,6 +6225,12 @@
       <c r="L121" t="n">
         <v>2</v>
       </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -5457,6 +6273,12 @@
       <c r="L122" t="n">
         <v>4</v>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -5495,6 +6317,12 @@
       <c r="L123" t="n">
         <v>2</v>
       </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -5537,6 +6365,12 @@
       <c r="L124" t="n">
         <v>1</v>
       </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -5575,6 +6409,12 @@
       <c r="L125" t="n">
         <v>2</v>
       </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -5613,6 +6453,12 @@
       <c r="L126" t="n">
         <v>2</v>
       </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -5651,6 +6497,12 @@
       <c r="L127" t="n">
         <v>2</v>
       </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -5689,6 +6541,12 @@
       <c r="L128" t="n">
         <v>2</v>
       </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -5731,6 +6589,12 @@
       <c r="L129" t="n">
         <v>4</v>
       </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -5769,6 +6633,12 @@
       <c r="L130" t="n">
         <v>2</v>
       </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -5807,6 +6677,12 @@
       <c r="L131" t="n">
         <v>2</v>
       </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -5845,6 +6721,12 @@
       <c r="L132" t="n">
         <v>2</v>
       </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -5887,6 +6769,16 @@
       <c r="L133" t="n">
         <v>4</v>
       </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -5925,6 +6817,12 @@
       <c r="L134" t="n">
         <v>2</v>
       </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -5963,6 +6861,12 @@
       <c r="L135" t="n">
         <v>2</v>
       </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6001,6 +6905,12 @@
       <c r="L136" t="n">
         <v>2</v>
       </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6039,6 +6949,12 @@
       <c r="L137" t="n">
         <v>2</v>
       </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6077,6 +6993,12 @@
       <c r="L138" t="n">
         <v>2</v>
       </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -6119,6 +7041,12 @@
       <c r="L139" t="n">
         <v>4</v>
       </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -6157,6 +7085,12 @@
       <c r="L140" t="n">
         <v>2</v>
       </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6195,6 +7129,12 @@
       <c r="L141" t="n">
         <v>1</v>
       </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6237,6 +7177,12 @@
       <c r="L142" t="n">
         <v>4</v>
       </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6279,6 +7225,16 @@
       <c r="L143" t="n">
         <v>4</v>
       </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>Mixed by gender</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>Y (mixed by gender)</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -6317,6 +7273,12 @@
       <c r="L144" t="n">
         <v>2</v>
       </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -6359,6 +7321,12 @@
       <c r="L145" t="n">
         <v>4</v>
       </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -6401,6 +7369,12 @@
       <c r="L146" t="n">
         <v>4</v>
       </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -6443,6 +7417,12 @@
       <c r="L147" t="n">
         <v>4</v>
       </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6485,6 +7465,12 @@
       <c r="L148" t="n">
         <v>4</v>
       </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -6523,6 +7509,12 @@
       <c r="L149" t="n">
         <v>2</v>
       </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -6565,6 +7557,12 @@
       <c r="L150" t="n">
         <v>4</v>
       </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -6603,6 +7601,12 @@
       <c r="L151" t="n">
         <v>2</v>
       </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -6641,6 +7645,12 @@
       <c r="L152" t="n">
         <v>2</v>
       </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6683,6 +7693,12 @@
       <c r="L153" t="n">
         <v>4</v>
       </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6721,6 +7737,12 @@
       <c r="L154" t="n">
         <v>2</v>
       </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -6763,6 +7785,16 @@
       <c r="L155" t="n">
         <v>4</v>
       </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -6805,6 +7837,16 @@
       <c r="L156" t="n">
         <v>4</v>
       </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -6847,6 +7889,12 @@
       <c r="L157" t="n">
         <v>4</v>
       </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -6889,6 +7937,12 @@
       <c r="L158" t="n">
         <v>4</v>
       </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -6935,6 +7989,12 @@
       <c r="L159" t="n">
         <v>2</v>
       </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6981,6 +8041,12 @@
       <c r="L160" t="n">
         <v>2</v>
       </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -7023,6 +8089,12 @@
       <c r="L161" t="n">
         <v>4</v>
       </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -7061,6 +8133,12 @@
       <c r="L162" t="n">
         <v>2</v>
       </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -7099,6 +8177,12 @@
       <c r="L163" t="n">
         <v>1</v>
       </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -7137,6 +8221,12 @@
       <c r="L164" t="n">
         <v>1</v>
       </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -7175,6 +8265,12 @@
       <c r="L165" t="n">
         <v>1</v>
       </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -7217,6 +8313,12 @@
       <c r="L166" t="n">
         <v>4</v>
       </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -7255,6 +8357,16 @@
       <c r="L167" t="n">
         <v>2</v>
       </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -7292,6 +8404,16 @@
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="n">
         <v>2</v>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="169">
@@ -7335,6 +8457,16 @@
       <c r="L169" t="n">
         <v>4</v>
       </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -7377,6 +8509,12 @@
       <c r="L170" t="n">
         <v>4</v>
       </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -7419,6 +8557,16 @@
       <c r="L171" t="n">
         <v>4</v>
       </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -7461,6 +8609,12 @@
       <c r="L172" t="n">
         <v>6</v>
       </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -7503,6 +8657,12 @@
       <c r="L173" t="n">
         <v>6</v>
       </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -7545,6 +8705,12 @@
       <c r="L174" t="n">
         <v>4</v>
       </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -7587,6 +8753,12 @@
       <c r="L175" t="n">
         <v>4</v>
       </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -7625,6 +8797,12 @@
       <c r="L176" t="n">
         <v>2</v>
       </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -7663,6 +8841,12 @@
       <c r="L177" t="n">
         <v>2</v>
       </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -7701,6 +8885,12 @@
       <c r="L178" t="n">
         <v>2</v>
       </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -7739,6 +8929,12 @@
       <c r="L179" t="n">
         <v>2</v>
       </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -7777,6 +8973,12 @@
       <c r="L180" t="n">
         <v>2</v>
       </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -7819,6 +9021,12 @@
       <c r="L181" t="n">
         <v>4</v>
       </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -7857,6 +9065,12 @@
       <c r="L182" t="n">
         <v>2</v>
       </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -7895,6 +9109,12 @@
       <c r="L183" t="n">
         <v>2</v>
       </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -7933,6 +9153,12 @@
       <c r="L184" t="n">
         <v>2</v>
       </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -7971,6 +9197,16 @@
       <c r="L185" t="n">
         <v>2</v>
       </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -8008,6 +9244,16 @@
       <c r="K186" t="inlineStr"/>
       <c r="L186" t="n">
         <v>2</v>
+      </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="187">
@@ -8051,6 +9297,12 @@
       <c r="L187" t="n">
         <v>4</v>
       </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -8089,6 +9341,12 @@
       <c r="L188" t="n">
         <v>2</v>
       </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -8127,6 +9385,12 @@
       <c r="L189" t="n">
         <v>2</v>
       </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -8169,6 +9433,12 @@
       <c r="L190" t="n">
         <v>4</v>
       </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -8211,6 +9481,12 @@
       <c r="L191" t="n">
         <v>4</v>
       </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -8253,6 +9529,12 @@
       <c r="L192" t="n">
         <v>4</v>
       </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -8295,6 +9577,12 @@
       <c r="L193" t="n">
         <v>4</v>
       </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -8333,6 +9621,12 @@
       <c r="L194" t="n">
         <v>2</v>
       </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -8371,6 +9665,12 @@
       <c r="L195" t="n">
         <v>2</v>
       </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -8413,6 +9713,12 @@
       <c r="L196" t="n">
         <v>4</v>
       </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -8455,6 +9761,12 @@
       <c r="L197" t="n">
         <v>4</v>
       </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -8493,6 +9805,12 @@
       <c r="L198" t="n">
         <v>2</v>
       </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -8531,6 +9849,12 @@
       <c r="L199" t="n">
         <v>2</v>
       </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -8569,6 +9893,12 @@
       <c r="L200" t="n">
         <v>2</v>
       </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -8607,6 +9937,12 @@
       <c r="L201" t="n">
         <v>2</v>
       </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -8645,6 +9981,12 @@
       <c r="L202" t="n">
         <v>2</v>
       </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -8683,6 +10025,12 @@
       <c r="L203" t="n">
         <v>2</v>
       </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr"/>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -8721,6 +10069,12 @@
       <c r="L204" t="n">
         <v>2</v>
       </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -8759,6 +10113,12 @@
       <c r="L205" t="n">
         <v>2</v>
       </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -8805,6 +10165,12 @@
       <c r="L206" t="n">
         <v>2</v>
       </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -8847,6 +10213,12 @@
       <c r="L207" t="n">
         <v>2</v>
       </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -8889,6 +10261,12 @@
       <c r="L208" t="n">
         <v>2</v>
       </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -8931,6 +10309,12 @@
       <c r="L209" t="n">
         <v>2</v>
       </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -8973,6 +10357,12 @@
       <c r="L210" t="n">
         <v>2</v>
       </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -9015,6 +10405,12 @@
       <c r="L211" t="n">
         <v>2</v>
       </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -9057,6 +10453,12 @@
       <c r="L212" t="n">
         <v>2</v>
       </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -9099,6 +10501,12 @@
       <c r="L213" t="n">
         <v>2</v>
       </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -9137,6 +10545,12 @@
       <c r="L214" t="n">
         <v>1</v>
       </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -9179,6 +10593,12 @@
       <c r="L215" t="n">
         <v>2</v>
       </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -9221,6 +10641,12 @@
       <c r="L216" t="n">
         <v>2</v>
       </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr"/>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -9263,6 +10689,12 @@
       <c r="L217" t="n">
         <v>2</v>
       </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr"/>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -9305,6 +10737,12 @@
       <c r="L218" t="n">
         <v>4</v>
       </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -9347,6 +10785,12 @@
       <c r="L219" t="n">
         <v>4</v>
       </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -9389,6 +10833,12 @@
       <c r="L220" t="n">
         <v>4</v>
       </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -9431,6 +10881,12 @@
       <c r="L221" t="n">
         <v>4</v>
       </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -9468,6 +10924,16 @@
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="n">
         <v>2</v>
+      </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
       </c>
     </row>
     <row r="223">
@@ -9511,6 +10977,12 @@
       <c r="L223" t="n">
         <v>4</v>
       </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -9553,6 +11025,12 @@
       <c r="L224" t="n">
         <v>4</v>
       </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -9591,6 +11069,12 @@
       <c r="L225" t="n">
         <v>2</v>
       </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -9629,6 +11113,12 @@
       <c r="L226" t="n">
         <v>2</v>
       </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -9671,6 +11161,12 @@
       <c r="L227" t="n">
         <v>1</v>
       </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -9713,6 +11209,12 @@
       <c r="L228" t="n">
         <v>1</v>
       </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -9755,6 +11257,12 @@
       <c r="L229" t="n">
         <v>1</v>
       </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -9793,6 +11301,12 @@
       <c r="L230" t="n">
         <v>2</v>
       </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -9839,6 +11353,12 @@
       <c r="L231" t="n">
         <v>2</v>
       </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -9881,6 +11401,12 @@
       <c r="L232" t="n">
         <v>3</v>
       </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -9919,6 +11445,12 @@
       <c r="L233" t="n">
         <v>2</v>
       </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -9961,6 +11493,12 @@
       <c r="L234" t="n">
         <v>4</v>
       </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -10003,6 +11541,16 @@
       <c r="L235" t="n">
         <v>4</v>
       </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -10045,6 +11593,12 @@
       <c r="L236" t="n">
         <v>1</v>
       </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -10083,6 +11637,12 @@
       <c r="L237" t="n">
         <v>2</v>
       </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -10121,6 +11681,12 @@
       <c r="L238" t="n">
         <v>2</v>
       </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -10163,6 +11729,12 @@
       <c r="L239" t="n">
         <v>1</v>
       </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -10201,6 +11773,12 @@
       <c r="L240" t="n">
         <v>2</v>
       </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -10243,6 +11821,12 @@
       <c r="L241" t="n">
         <v>1</v>
       </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -10285,6 +11869,12 @@
       <c r="L242" t="n">
         <v>4</v>
       </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -10323,6 +11913,12 @@
       <c r="L243" t="n">
         <v>2</v>
       </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -10361,6 +11957,12 @@
       <c r="L244" t="n">
         <v>1</v>
       </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr"/>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -10399,6 +12001,12 @@
       <c r="L245" t="n">
         <v>2</v>
       </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr"/>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -10437,6 +12045,12 @@
       <c r="L246" t="n">
         <v>2</v>
       </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr"/>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -10479,6 +12093,16 @@
       <c r="L247" t="n">
         <v>4</v>
       </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -10521,6 +12145,12 @@
       <c r="L248" t="n">
         <v>4</v>
       </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -10563,6 +12193,12 @@
       <c r="L249" t="n">
         <v>4</v>
       </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr"/>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -10601,6 +12237,12 @@
       <c r="L250" t="n">
         <v>2</v>
       </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -10639,6 +12281,12 @@
       <c r="L251" t="n">
         <v>2</v>
       </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr"/>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -10677,6 +12325,12 @@
       <c r="L252" t="n">
         <v>2</v>
       </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr"/>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -10719,6 +12373,12 @@
       <c r="L253" t="n">
         <v>2</v>
       </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr"/>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -10761,6 +12421,12 @@
       <c r="L254" t="n">
         <v>2</v>
       </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr"/>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -10803,6 +12469,12 @@
       <c r="L255" t="n">
         <v>2</v>
       </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr"/>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -10845,6 +12517,12 @@
       <c r="L256" t="n">
         <v>2</v>
       </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr"/>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -10883,6 +12561,12 @@
       <c r="L257" t="n">
         <v>1</v>
       </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr"/>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -10925,6 +12609,12 @@
       <c r="L258" t="n">
         <v>2</v>
       </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr"/>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -10963,9 +12653,15 @@
       <c r="L259" t="n">
         <v>1</v>
       </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>Not in legacy portfolio</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L259"/>
+  <autoFilter ref="A1:N259"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10976,7 +12672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -11043,6 +12739,30 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Legacy Core Assortment FW27</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>A pre-Tobias-data flag already in the SS26 tiering workbook (57/1,860 Base+Gender rows = 'Yes') -- sparse and partial, not a full FW27 range list. Rolled up to Base grain here (Yes if either gender was Yes); 2 bases are genuinely 'Mixed by gender'. 'Not in legacy portfolio' means this franchise's base name has no match in the 1,860-row tiering sheet (new, renamed, or a naming mismatch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Agrees with new FW27-active?</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>'Core Assortment FW27' is a narrow strategic-item flag (57/1,860 bases), not a full range flag -- most franchises are legitimately 'No' and still Active in FW27, so that's NOT a disagreement and this column is left blank for 'No'/'Not in legacy portfolio' rows. Only computed where the legacy flag said Yes/Mixed: 'N' rows are the ones worth a second look -- a franchise previously flagged core for FW27 that no longer shows Active there in the new data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Simplify Core Assortment columns: plain FW27 Yes/No, SS28 To confirm
Drops the historic-sales/legacy-portfolio cross-check framing for now --
that comparison belongs in a later step once updated sales data is in.
Core Assortment FW27 is now a plain Yes/No rollup of the existing tiering
workbook flag; Core Assortment SS28 has no source yet and is marked "To
confirm" for every row.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bz4WiqJXGrQWfCc7f9Cm8G
</commit_message>
<xml_diff>
--- a/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
+++ b/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
@@ -444,8 +444,8 @@
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="29" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -511,12 +511,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Legacy Core Assortment FW27</t>
+          <t>Core Assortment FW27</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Agrees with new FW27-active?</t>
+          <t>Core Assortment SS28</t>
         </is>
       </c>
     </row>
@@ -559,10 +559,14 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -608,7 +612,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -660,7 +664,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -710,7 +714,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -754,7 +762,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -798,7 +810,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -839,10 +855,14 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -886,7 +906,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -934,7 +958,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -978,7 +1006,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1022,7 +1054,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1063,10 +1099,14 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N13" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1110,7 +1150,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1154,7 +1198,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1202,7 +1250,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1243,10 +1295,14 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1290,7 +1346,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1331,10 +1391,14 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1378,7 +1442,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1422,7 +1490,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1466,7 +1538,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1520,7 +1596,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1568,7 +1648,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1609,10 +1693,14 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1660,7 +1748,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1705,10 +1797,14 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N27" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1756,7 +1852,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1804,7 +1904,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1852,7 +1956,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1900,7 +2008,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1948,7 +2060,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1996,7 +2112,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2044,7 +2164,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2092,7 +2216,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2137,10 +2265,14 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2192,7 +2324,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2242,7 +2378,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -2294,7 +2430,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -2344,7 +2480,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2389,10 +2529,14 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N41" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2440,7 +2584,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2488,7 +2636,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2536,7 +2688,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2584,7 +2740,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2634,7 +2794,7 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2844,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2732,7 +2896,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2780,7 +2948,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2828,7 +3000,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2873,10 +3049,14 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N51" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2920,7 +3100,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2964,7 +3148,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3008,7 +3196,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3049,10 +3241,14 @@
       </c>
       <c r="M55" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N55" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3100,7 +3296,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3150,7 +3350,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -3202,7 +3402,7 @@
       </c>
       <c r="N58" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -3252,7 +3452,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3300,7 +3504,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3348,7 +3556,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N61" t="inlineStr"/>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3400,7 +3612,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3452,7 +3668,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3502,7 +3722,7 @@
       </c>
       <c r="N64" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -3558,7 +3778,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3828,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3656,7 +3880,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3704,7 +3932,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3752,7 +3984,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3800,7 +4036,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3848,7 +4088,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3896,7 +4140,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr"/>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3944,7 +4192,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3989,10 +4241,14 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4040,7 +4296,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4088,7 +4348,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N76" t="inlineStr"/>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4136,7 +4400,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4184,7 +4452,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4229,10 +4501,14 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N79" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4277,10 +4553,14 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N80" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4325,10 +4605,14 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N81" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4372,7 +4656,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N82" t="inlineStr"/>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4417,10 +4705,14 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N83" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4465,10 +4757,14 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N84" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4512,7 +4808,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N85" t="inlineStr"/>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4562,7 +4862,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4912,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N87" t="inlineStr"/>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4660,7 +4964,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N88" t="inlineStr"/>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -4708,7 +5016,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N89" t="inlineStr"/>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -4759,10 +5071,14 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N90" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -4807,10 +5123,14 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N91" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -4854,7 +5174,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N92" t="inlineStr"/>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -4898,7 +5222,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N93" t="inlineStr"/>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -4946,7 +5274,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N94" t="inlineStr"/>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -4996,7 +5328,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5048,7 +5380,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5091,10 +5423,14 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N97" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5138,7 +5474,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5183,10 +5523,14 @@
       </c>
       <c r="M99" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N99" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5227,10 +5571,14 @@
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N100" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5280,7 +5628,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5330,7 +5678,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N102" t="inlineStr"/>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5375,10 +5727,14 @@
       </c>
       <c r="M103" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N103" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5428,7 +5784,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5480,7 +5836,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5882,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N106" t="inlineStr"/>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5570,7 +5930,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N107" t="inlineStr"/>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -5620,7 +5984,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5668,7 +6032,7 @@
       </c>
       <c r="N109" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5716,7 +6080,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5759,12 +6123,12 @@
       </c>
       <c r="M111" t="inlineStr">
         <is>
-          <t>Mixed by gender</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
         <is>
-          <t>Y (mixed by gender)</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -5810,7 +6174,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N112" t="inlineStr"/>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5854,7 +6222,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N113" t="inlineStr"/>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -5898,7 +6270,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N114" t="inlineStr"/>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -5948,7 +6324,7 @@
       </c>
       <c r="N115" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -6000,7 +6376,7 @@
       </c>
       <c r="N116" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -6046,7 +6422,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N117" t="inlineStr"/>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6091,10 +6471,14 @@
       </c>
       <c r="M118" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N118" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6142,7 +6526,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N119" t="inlineStr"/>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6183,10 +6571,14 @@
       </c>
       <c r="M120" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N120" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6227,10 +6619,14 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N121" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6278,7 +6674,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N122" t="inlineStr"/>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6322,7 +6722,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N123" t="inlineStr"/>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6367,10 +6771,14 @@
       </c>
       <c r="M124" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N124" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6414,7 +6822,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N125" t="inlineStr"/>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -6458,7 +6870,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N126" t="inlineStr"/>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6502,7 +6918,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N127" t="inlineStr"/>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6543,10 +6963,14 @@
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N128" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6594,7 +7018,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N129" t="inlineStr"/>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6638,7 +7066,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N130" t="inlineStr"/>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6682,7 +7114,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N131" t="inlineStr"/>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6726,7 +7162,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N132" t="inlineStr"/>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6776,7 +7216,7 @@
       </c>
       <c r="N133" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -6819,10 +7259,14 @@
       </c>
       <c r="M134" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N134" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -6866,7 +7310,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N135" t="inlineStr"/>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -6910,7 +7358,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N136" t="inlineStr"/>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -6954,7 +7406,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N137" t="inlineStr"/>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -6998,7 +7454,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N138" t="inlineStr"/>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7046,7 +7506,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N139" t="inlineStr"/>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7087,10 +7551,14 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N140" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7131,10 +7599,14 @@
       </c>
       <c r="M141" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N141" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7179,10 +7651,14 @@
       </c>
       <c r="M142" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N142" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -7227,12 +7703,12 @@
       </c>
       <c r="M143" t="inlineStr">
         <is>
-          <t>Mixed by gender</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="N143" t="inlineStr">
         <is>
-          <t>Y (mixed by gender)</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -7278,7 +7754,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N144" t="inlineStr"/>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -7326,7 +7806,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N145" t="inlineStr"/>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -7374,7 +7858,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N146" t="inlineStr"/>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -7422,7 +7910,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N147" t="inlineStr"/>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -7470,7 +7962,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N148" t="inlineStr"/>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -7511,10 +8007,14 @@
       </c>
       <c r="M149" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N149" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -7562,7 +8062,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N150" t="inlineStr"/>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -7606,7 +8110,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -7647,10 +8155,14 @@
       </c>
       <c r="M152" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N152" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -7698,7 +8210,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N153" t="inlineStr"/>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -7742,7 +8258,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N154" t="inlineStr"/>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -7792,7 +8312,7 @@
       </c>
       <c r="N155" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -7844,7 +8364,7 @@
       </c>
       <c r="N156" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -7894,7 +8414,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N157" t="inlineStr"/>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -7942,7 +8466,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr"/>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -7991,10 +8519,14 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N159" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -8043,10 +8575,14 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N160" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -8094,7 +8630,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N161" t="inlineStr"/>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -8138,7 +8678,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N162" t="inlineStr"/>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -8179,10 +8723,14 @@
       </c>
       <c r="M163" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N163" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -8223,10 +8771,14 @@
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N164" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -8267,10 +8819,14 @@
       </c>
       <c r="M165" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N165" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -8318,7 +8874,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N166" t="inlineStr"/>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -8364,7 +8924,7 @@
       </c>
       <c r="N167" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -8412,7 +8972,7 @@
       </c>
       <c r="N168" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -8464,7 +9024,7 @@
       </c>
       <c r="N169" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -8514,7 +9074,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N170" t="inlineStr"/>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -8564,7 +9128,7 @@
       </c>
       <c r="N171" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -8611,10 +9175,14 @@
       </c>
       <c r="M172" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N172" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -8659,10 +9227,14 @@
       </c>
       <c r="M173" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N173" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -8710,7 +9282,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N174" t="inlineStr"/>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -8758,7 +9334,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N175" t="inlineStr"/>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -8802,7 +9382,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N176" t="inlineStr"/>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -8846,7 +9430,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N177" t="inlineStr"/>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -8887,10 +9475,14 @@
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N178" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -8931,10 +9523,14 @@
       </c>
       <c r="M179" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N179" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -8978,7 +9574,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N180" t="inlineStr"/>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -9026,7 +9626,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N181" t="inlineStr"/>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -9070,7 +9674,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N182" t="inlineStr"/>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9111,10 +9719,14 @@
       </c>
       <c r="M183" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N183" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -9155,10 +9767,14 @@
       </c>
       <c r="M184" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N184" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -9204,7 +9820,7 @@
       </c>
       <c r="N185" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -9252,7 +9868,7 @@
       </c>
       <c r="N186" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -9299,10 +9915,14 @@
       </c>
       <c r="M187" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N187" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -9346,7 +9966,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N188" t="inlineStr"/>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -9390,7 +10014,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N189" t="inlineStr"/>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -9435,10 +10063,14 @@
       </c>
       <c r="M190" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N190" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -9486,7 +10118,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N191" t="inlineStr"/>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -9534,7 +10170,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N192" t="inlineStr"/>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -9582,7 +10222,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N193" t="inlineStr"/>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -9623,10 +10267,14 @@
       </c>
       <c r="M194" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N194" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -9667,10 +10315,14 @@
       </c>
       <c r="M195" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N195" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -9715,10 +10367,14 @@
       </c>
       <c r="M196" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N196" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -9766,7 +10422,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N197" t="inlineStr"/>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -9807,10 +10467,14 @@
       </c>
       <c r="M198" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N198" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -9851,10 +10515,14 @@
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N199" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -9898,7 +10566,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N200" t="inlineStr"/>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -9942,7 +10614,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N201" t="inlineStr"/>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -9986,7 +10662,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N202" t="inlineStr"/>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -10030,7 +10710,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N203" t="inlineStr"/>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -10074,7 +10758,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N204" t="inlineStr"/>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -10118,7 +10806,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N205" t="inlineStr"/>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -10170,7 +10862,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N206" t="inlineStr"/>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -10218,7 +10914,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N207" t="inlineStr"/>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -10266,7 +10966,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N208" t="inlineStr"/>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -10314,7 +11018,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N209" t="inlineStr"/>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -10362,7 +11070,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N210" t="inlineStr"/>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -10410,7 +11122,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N211" t="inlineStr"/>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -10458,7 +11174,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N212" t="inlineStr"/>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -10506,7 +11226,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N213" t="inlineStr"/>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -10550,7 +11274,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N214" t="inlineStr"/>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -10598,7 +11326,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N215" t="inlineStr"/>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -10646,7 +11378,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N216" t="inlineStr"/>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -10694,7 +11430,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N217" t="inlineStr"/>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -10739,10 +11479,14 @@
       </c>
       <c r="M218" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N218" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -10787,10 +11531,14 @@
       </c>
       <c r="M219" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N219" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -10838,7 +11586,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N220" t="inlineStr"/>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -10886,7 +11638,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N221" t="inlineStr"/>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -10932,7 +11688,7 @@
       </c>
       <c r="N222" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -10982,7 +11738,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N223" t="inlineStr"/>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -11030,7 +11790,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N224" t="inlineStr"/>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -11074,7 +11838,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N225" t="inlineStr"/>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -11118,7 +11886,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N226" t="inlineStr"/>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -11163,10 +11935,14 @@
       </c>
       <c r="M227" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N227" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -11214,7 +11990,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N228" t="inlineStr"/>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -11262,7 +12042,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N229" t="inlineStr"/>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -11303,10 +12087,14 @@
       </c>
       <c r="M230" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N230" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -11358,7 +12146,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N231" t="inlineStr"/>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -11406,7 +12198,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N232" t="inlineStr"/>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -11450,7 +12246,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N233" t="inlineStr"/>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -11498,7 +12298,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N234" t="inlineStr"/>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -11548,7 +12352,7 @@
       </c>
       <c r="N235" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -11598,7 +12402,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N236" t="inlineStr"/>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -11642,7 +12450,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N237" t="inlineStr"/>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -11686,7 +12498,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N238" t="inlineStr"/>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -11734,7 +12550,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N239" t="inlineStr"/>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -11778,7 +12598,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N240" t="inlineStr"/>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -11826,7 +12650,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N241" t="inlineStr"/>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -11871,10 +12699,14 @@
       </c>
       <c r="M242" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N242" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -11915,10 +12747,14 @@
       </c>
       <c r="M243" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N243" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -11959,10 +12795,14 @@
       </c>
       <c r="M244" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N244" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -12006,7 +12846,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N245" t="inlineStr"/>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -12050,7 +12894,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N246" t="inlineStr"/>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -12100,7 +12948,7 @@
       </c>
       <c r="N247" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>To confirm</t>
         </is>
       </c>
     </row>
@@ -12147,10 +12995,14 @@
       </c>
       <c r="M248" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N248" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -12198,7 +13050,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N249" t="inlineStr"/>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -12239,10 +13095,14 @@
       </c>
       <c r="M250" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N250" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -12283,10 +13143,14 @@
       </c>
       <c r="M251" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N251" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -12327,10 +13191,14 @@
       </c>
       <c r="M252" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N252" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -12378,7 +13246,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N253" t="inlineStr"/>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -12426,7 +13298,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N254" t="inlineStr"/>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -12471,10 +13347,14 @@
       </c>
       <c r="M255" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N255" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -12519,10 +13399,14 @@
       </c>
       <c r="M256" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N256" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -12566,7 +13450,11 @@
           <t>No</t>
         </is>
       </c>
-      <c r="N257" t="inlineStr"/>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -12611,10 +13499,14 @@
       </c>
       <c r="M258" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N258" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -12655,10 +13547,14 @@
       </c>
       <c r="M259" t="inlineStr">
         <is>
-          <t>Not in legacy portfolio</t>
-        </is>
-      </c>
-      <c r="N259" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>To confirm</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N259"/>
@@ -12742,24 +13638,24 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Legacy Core Assortment FW27</t>
+          <t>Core Assortment FW27</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>A pre-Tobias-data flag already in the SS26 tiering workbook (57/1,860 Base+Gender rows = 'Yes') -- sparse and partial, not a full FW27 range list. Rolled up to Base grain here (Yes if either gender was Yes); 2 bases are genuinely 'Mixed by gender'. 'Not in legacy portfolio' means this franchise's base name has no match in the 1,860-row tiering sheet (new, renamed, or a naming mismatch).</t>
+          <t>Yes/No, from the flag already in the SS26 tiering workbook (57/1,860 Base+Gender rows = 'Yes'), rolled up to Base grain (Yes if either gender was Yes).</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Agrees with new FW27-active?</t>
+          <t>Core Assortment SS28</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>'Core Assortment FW27' is a narrow strategic-item flag (57/1,860 bases), not a full range flag -- most franchises are legitimately 'No' and still Active in FW27, so that's NOT a disagreement and this column is left blank for 'No'/'Not in legacy portfolio' rows. Only computed where the legacy flag said Yes/Mixed: 'N' rows are the ones worth a second look -- a franchise previously flagged core for FW27 that no longer shows Active there in the new data.</t>
+          <t>No source yet -- the flag was only ever defined for FW27. Left as 'To confirm' for every row until Tobias/Isabelle define it for SS28.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add FW27 Pic Centric file, resolve margin target + images for all franchises
build_product_images.py now processes both FW27 and SS28 Pic Centric
workbooks into one combined gm_by_code.json (SS28 wins on the rare
conflict -- 213/215 overlapping codes agree exactly, the other 2 only
differ on RRP, not GM%). build_franchise_list.py's margin-target lookup
now uses the franchise's own representative code against this combined
file instead of an SS28-only lookup, with a same-franchise fallback.

RR-008 (margin target) and RR-015 (product images) move from
"SS28-resolved, FW27-open" to fully resolved: all 258 franchises now
have Margin target filled (up from 198), and the image repository covers
496/500 combined codes (up from 334/336 SS28-only).
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bz4WiqJXGrQWfCc7f9Cm8G
</commit_message>
<xml_diff>
--- a/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
+++ b/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
@@ -629,7 +629,9 @@
           <t>Everyday Outdoor; Freeride Ski &amp; Snowboard; Skitouring; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>65</v>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>1</v>
@@ -719,7 +721,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>61.3</v>
+      </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>1</v>
@@ -1465,7 +1469,9 @@
           <t>Mountaineering / Alpinism; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>61</v>
+      </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="n">
         <v>1</v>
@@ -1555,7 +1561,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>64</v>
+      </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="n">
         <v>1</v>
@@ -1645,7 +1653,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>74.3</v>
+      </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="n">
         <v>1</v>
@@ -1735,7 +1745,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>61.3</v>
+      </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="n">
         <v>1</v>
@@ -2089,7 +2101,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>61.3</v>
+      </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="n">
         <v>1</v>
@@ -2179,7 +2193,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>62</v>
+      </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="n">
         <v>1</v>
@@ -2269,7 +2285,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>62</v>
+      </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="n">
         <v>1</v>
@@ -2359,7 +2377,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>61.3</v>
+      </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="n">
         <v>1</v>
@@ -2449,7 +2469,9 @@
           <t>Everyday Outdoor; Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>60</v>
+      </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="n">
         <v>1</v>
@@ -5425,7 +5447,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing; Skitouring; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="n">
+        <v>64</v>
+      </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="n">
         <v>2</v>
@@ -5515,7 +5539,9 @@
           <t>Everyday Outdoor; Freeride Ski &amp; Snowboard; Resort Skiing; Skitouring; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="n">
+        <v>57</v>
+      </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="n">
         <v>2</v>
@@ -5605,7 +5631,9 @@
           <t>Freeride Ski &amp; Snowboard; Mountaineering / Alpinism; Resort Skiing; Ski Mountaineering; Skitouring; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>60</v>
+      </c>
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="n">
         <v>2</v>
@@ -8399,7 +8427,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="n">
+        <v>60</v>
+      </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="n">
         <v>2</v>
@@ -8689,7 +8719,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="n">
         <v>2</v>
@@ -9385,7 +9417,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr"/>
+      <c r="K92" t="n">
+        <v>65</v>
+      </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="n">
         <v>2</v>
@@ -9475,7 +9509,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>61</v>
+      </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="n">
         <v>2</v>
@@ -9569,7 +9605,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="n">
+        <v>64</v>
+      </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="n">
         <v>1</v>
@@ -9947,7 +9985,9 @@
           <t>Fast Hiking; Skitouring; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr"/>
+      <c r="K98" t="n">
+        <v>60</v>
+      </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="n">
         <v>2</v>
@@ -10229,7 +10269,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="n">
+        <v>65.40000000000001</v>
+      </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="n">
         <v>1</v>
@@ -10323,7 +10365,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr"/>
+      <c r="K102" t="n">
+        <v>65.40000000000001</v>
+      </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="n">
         <v>1</v>
@@ -10713,7 +10757,9 @@
           <t>Freeride Ski &amp; Snowboard; Mountaineering / Alpinism; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr"/>
+      <c r="K106" t="n">
+        <v>61.5</v>
+      </c>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="n">
         <v>2</v>
@@ -10803,7 +10849,9 @@
           <t>Freeride Ski &amp; Snowboard; Mountaineering / Alpinism; Skitouring</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr"/>
+      <c r="K107" t="n">
+        <v>55</v>
+      </c>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="n">
         <v>2</v>
@@ -10993,7 +11041,9 @@
           <t>Mountaineering / Alpinism; Ski Mountaineering; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr"/>
+      <c r="K109" t="n">
+        <v>60</v>
+      </c>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="n">
         <v>2</v>
@@ -11083,7 +11133,9 @@
           <t>Mountaineering / Alpinism; Ski Mountaineering; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr"/>
+      <c r="K110" t="n">
+        <v>66</v>
+      </c>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="n">
         <v>2</v>
@@ -11173,7 +11225,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="n">
+        <v>61</v>
+      </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="n">
         <v>2</v>
@@ -11263,7 +11317,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr"/>
+      <c r="K112" t="n">
+        <v>60</v>
+      </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="n">
         <v>2</v>
@@ -11353,7 +11409,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr"/>
+      <c r="K113" t="n">
+        <v>61.5</v>
+      </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="n">
         <v>2</v>
@@ -11443,7 +11501,9 @@
           <t>Expeditions; Mountaineering / Alpinism; Ski Mountaineering</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr"/>
+      <c r="K114" t="n">
+        <v>55</v>
+      </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="n">
         <v>2</v>
@@ -13549,7 +13609,9 @@
           <t>Everyday Outdoor; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr"/>
+      <c r="K137" t="n">
+        <v>65</v>
+      </c>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="n">
         <v>2</v>
@@ -14191,7 +14253,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr"/>
+      <c r="K144" t="n">
+        <v>62.9</v>
+      </c>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="n">
         <v>2</v>
@@ -15149,7 +15213,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr"/>
+      <c r="K154" t="n">
+        <v>65</v>
+      </c>
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="n">
         <v>2</v>
@@ -15947,7 +16013,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing; Ski Mountaineering; Skitouring</t>
         </is>
       </c>
-      <c r="K162" t="inlineStr"/>
+      <c r="K162" t="n">
+        <v>62.9</v>
+      </c>
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="n">
         <v>2</v>
@@ -16037,7 +16105,9 @@
           <t>Freeride Ski &amp; Snowboard</t>
         </is>
       </c>
-      <c r="K163" t="inlineStr"/>
+      <c r="K163" t="n">
+        <v>59.3</v>
+      </c>
       <c r="L163" t="inlineStr"/>
       <c r="M163" t="n">
         <v>1</v>
@@ -16127,7 +16197,9 @@
           <t>Skitouring</t>
         </is>
       </c>
-      <c r="K164" t="inlineStr"/>
+      <c r="K164" t="n">
+        <v>52.2</v>
+      </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="n">
         <v>1</v>
@@ -16217,7 +16289,9 @@
           <t>Freeride Ski &amp; Snowboard</t>
         </is>
       </c>
-      <c r="K165" t="inlineStr"/>
+      <c r="K165" t="n">
+        <v>65</v>
+      </c>
       <c r="L165" t="inlineStr"/>
       <c r="M165" t="n">
         <v>1</v>
@@ -16403,7 +16477,9 @@
           <t>Mountaineering / Alpinism; Resort Skiing; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K167" t="inlineStr"/>
+      <c r="K167" t="n">
+        <v>60</v>
+      </c>
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="n">
         <v>2</v>
@@ -16493,7 +16569,9 @@
           <t>Mountaineering / Alpinism; Resort Skiing</t>
         </is>
       </c>
-      <c r="K168" t="inlineStr"/>
+      <c r="K168" t="n">
+        <v>60</v>
+      </c>
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="n">
         <v>2</v>
@@ -17279,7 +17357,9 @@
           <t>Everyday Outdoor; Fast Hiking; Trail Running; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K176" t="inlineStr"/>
+      <c r="K176" t="n">
+        <v>60</v>
+      </c>
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="n">
         <v>2</v>
@@ -17369,7 +17449,9 @@
           <t>Everyday Outdoor; Fast Hiking; Trail Running; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K177" t="inlineStr"/>
+      <c r="K177" t="n">
+        <v>60</v>
+      </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="n">
         <v>2</v>
@@ -17635,7 +17717,9 @@
           <t>Everyday Outdoor; Fast Hiking; Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K180" t="inlineStr"/>
+      <c r="K180" t="n">
+        <v>50</v>
+      </c>
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="n">
         <v>2</v>
@@ -18073,7 +18157,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K185" t="inlineStr"/>
+      <c r="K185" t="n">
+        <v>62</v>
+      </c>
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="n">
         <v>2</v>
@@ -18163,7 +18249,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K186" t="inlineStr"/>
+      <c r="K186" t="n">
+        <v>64</v>
+      </c>
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>2</v>
@@ -18353,7 +18441,9 @@
           <t>Freeride Ski &amp; Snowboard; Mountaineering / Alpinism; Skitouring</t>
         </is>
       </c>
-      <c r="K188" t="inlineStr"/>
+      <c r="K188" t="n">
+        <v>55</v>
+      </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="n">
         <v>2</v>
@@ -18443,7 +18533,9 @@
           <t>Freeride Ski &amp; Snowboard; Mountaineering / Alpinism; Skitouring</t>
         </is>
       </c>
-      <c r="K189" t="inlineStr"/>
+      <c r="K189" t="n">
+        <v>55</v>
+      </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>2</v>
@@ -18933,7 +19025,9 @@
           <t>Resort Skiing</t>
         </is>
       </c>
-      <c r="K194" t="inlineStr"/>
+      <c r="K194" t="n">
+        <v>60</v>
+      </c>
       <c r="L194" t="inlineStr"/>
       <c r="M194" t="n">
         <v>2</v>
@@ -19023,7 +19117,9 @@
           <t>Resort Skiing</t>
         </is>
       </c>
-      <c r="K195" t="inlineStr"/>
+      <c r="K195" t="n">
+        <v>60</v>
+      </c>
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="n">
         <v>2</v>
@@ -19313,7 +19409,9 @@
           <t>Resort Skiing</t>
         </is>
       </c>
-      <c r="K198" t="inlineStr"/>
+      <c r="K198" t="n">
+        <v>62</v>
+      </c>
       <c r="L198" t="inlineStr"/>
       <c r="M198" t="n">
         <v>2</v>
@@ -19403,7 +19501,9 @@
           <t>Resort Skiing</t>
         </is>
       </c>
-      <c r="K199" t="inlineStr"/>
+      <c r="K199" t="n">
+        <v>63</v>
+      </c>
       <c r="L199" t="inlineStr"/>
       <c r="M199" t="n">
         <v>2</v>
@@ -19493,7 +19593,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K200" t="inlineStr"/>
+      <c r="K200" t="n">
+        <v>55</v>
+      </c>
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="n">
         <v>2</v>
@@ -19583,7 +19685,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing; Skitouring</t>
         </is>
       </c>
-      <c r="K201" t="inlineStr"/>
+      <c r="K201" t="n">
+        <v>59.2</v>
+      </c>
       <c r="L201" t="inlineStr"/>
       <c r="M201" t="n">
         <v>2</v>
@@ -19673,7 +19777,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K202" t="inlineStr"/>
+      <c r="K202" t="n">
+        <v>59.2</v>
+      </c>
       <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>2</v>
@@ -19763,7 +19869,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing</t>
         </is>
       </c>
-      <c r="K203" t="inlineStr"/>
+      <c r="K203" t="n">
+        <v>59.2</v>
+      </c>
       <c r="L203" t="inlineStr"/>
       <c r="M203" t="n">
         <v>2</v>
@@ -19853,7 +19961,9 @@
           <t>Freeride Ski &amp; Snowboard; Resort Skiing; Skitouring</t>
         </is>
       </c>
-      <c r="K204" t="inlineStr"/>
+      <c r="K204" t="n">
+        <v>59.2</v>
+      </c>
       <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>2</v>
@@ -19943,7 +20053,9 @@
           <t>Everyday Outdoor</t>
         </is>
       </c>
-      <c r="K205" t="inlineStr"/>
+      <c r="K205" t="n">
+        <v>57</v>
+      </c>
       <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>2</v>
@@ -20837,7 +20949,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K214" t="inlineStr"/>
+      <c r="K214" t="n">
+        <v>52.2</v>
+      </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="n">
         <v>1</v>
@@ -21627,7 +21741,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K222" t="inlineStr"/>
+      <c r="K222" t="n">
+        <v>60</v>
+      </c>
       <c r="L222" t="inlineStr"/>
       <c r="M222" t="n">
         <v>2</v>
@@ -24925,7 +25041,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K257" t="inlineStr"/>
+      <c r="K257" t="n">
+        <v>0</v>
+      </c>
       <c r="L257" t="inlineStr"/>
       <c r="M257" t="n">
         <v>1</v>
@@ -25107,7 +25225,9 @@
           <t>Trekking / Hiking</t>
         </is>
       </c>
-      <c r="K259" t="inlineStr"/>
+      <c r="K259" t="n">
+        <v>59.8</v>
+      </c>
       <c r="L259" t="inlineStr"/>
       <c r="M259" t="n">
         <v>1</v>
@@ -25235,7 +25355,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Target GM0% from the SS28 'Pic Centric' workbook -- the FW27/SS28 range files themselves have no margin field (RR-008). SS28-only for now; blank for franchises with no SS28 code until an equivalent FW27 file arrives.</t>
+          <t>Target GM0% from the FW27+SS28 'Pic Centric' workbooks -- the FW27/SS28 range files themselves have no margin field (RR-008). Blank only for franchises with no Pic Centric match in either season.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename "Margin target" to "Target GM0%" for clarity vs. Forecast GP%
User asked to clarify the distinction between GP% (a forecast outcome,
from FC3 volume/price/channel mix) and the margin figure pulled from the
Pic Centric files (a pricing/costing goal, independent of the sales
forecast) -- renaming the column/label to match the source field name
exactly, rather than the generic "Margin target", makes that clearer at
a glance. Documents the distinction in RR-008 and the franchise list's
Notes sheet. Also logs 2025/2026 actual sales figures as a future Next
Steps item once that data arrives.
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Bz4WiqJXGrQWfCc7f9Cm8G
</commit_message>
<xml_diff>
--- a/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
+++ b/data/range_review/outputs/FW27_SS28_Franchise_Review_List.xlsx
@@ -442,7 +442,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="45" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
@@ -513,7 +513,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Margin target</t>
+          <t>Target GM0%</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -25350,12 +25350,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Margin target</t>
+          <t>Target GM0%</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Target GM0% from the FW27+SS28 'Pic Centric' workbooks -- the FW27/SS28 range files themselves have no margin field (RR-008). Blank only for franchises with no Pic Centric match in either season.</t>
+          <t>A pricing/costing GOAL set during product costing (Target RRP vs. Target FOB), from the FW27+SS28 'Pic Centric' workbooks -- the FW27/SS28 range files themselves have no margin field (RR-008). NOT the same thing as Forecast GP% (the Forecast sheet/page's blended/DTC/Wholesale GP% columns), which is a forecast OUTCOME derived from FC3 volume, price and channel mix -- the two can genuinely differ, and the gap is itself worth a look. Blank only for franchises with no Pic Centric match in either season.</t>
         </is>
       </c>
     </row>

</xml_diff>